<commit_message>
v4.2: reply with two boxes, review + merch-sensei build feasibility
build_review.py now prints a second box in merch-sensei's format (AUTH, ORDER,
IDEMPOTENCY, ADDRESS, STATUS MAP, WEBHOOK, POLLING, PRE-CONFIRM FAIL, TRACKING,
CANCEL/RETURNS, CATALOG, BALANCE, sandbox run, complexity, risks, build files,
checklist, notes, handoff). Lines come from tech.feasibility or are derived
from the checks. The Tech tab starts with the same table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/printstop/Printstop_Review.xlsx
+++ b/examples/printstop/Printstop_Review.xlsx
@@ -3343,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3384,7 +3384,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Endpoints</t>
+          <t>Build feasibility (merch-sensei format)</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
@@ -3393,862 +3393,1092 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Operation</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Token</t>
+          <t>AUTH</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>GET ?method=generate_token&amp;corporate_id={id}</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Headers client-secret, client-id, user-name. TTL not documented.</t>
+          <t>JWT via GET generate_token → tokens table (credentials under one key "printstop"). TTL not documented. Every call also needs client-id and client-secret headers.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Place order</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>POST ?method=order</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>profile, product, shipping (or location code), billing code. 200 orders_id; 409 {orders:[ids]} keyed on user; 400/401/500.</t>
+          <t>POST method=order → orders_id. Async (In Production after) → iswebhookConfiration true. code/apiOrderId/addedBy contract OK.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Track order</t>
+          <t>IDEMPOTENCY</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>POST ?method=order_status&amp;orders_id={id}</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>orders_status (same field our polling reads), tracking_number, tracking_url, shipping_company, due and delivery dates.</t>
+          <t>reference_number optional, not echoed, not searchable. 409 is keyed on the user, so never auto-link via callVendorRefetch.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>ADDRESS</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>POST ?method=product_listing</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>total + data[product_id, name, status]. No paging.</t>
+          <t>shipping_* fields map. Recipient name/phone go in profile (shipping has no name). company_name, corporate_id constants. Country 99 = India only.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Product details</t>
+          <t>STATUS MAP</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>POST ?method=product_details</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Selector not documented (assume &amp;product_id=). Sizes, templates, images, GST, HSN. No price.</t>
+          <t>Only "in production" → CONFIRMED known. Full list needed.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Categories</t>
+          <t>WEBHOOK</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>POST ?method=category_listing</t>
+          <t>➖</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Category names for products.</t>
+          <t>None. Polling only; nothing to add in plumAuth.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Create user</t>
+          <t>POLLING</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>POST ?method=create_user&amp;...</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>All data in the URL query. Only needed if orders require an existing user.</t>
+          <t>order_status returns top-level orders_status (the field the base reads). Add id to merchandiseOrderTrackingVendorIds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>PRE-CONFIRM FAIL</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Not documented whether an accepted order can be rejected (approval workflow exists in create_user).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Order field mapping</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>tracking_number, tracking_url, shipping_company, orders_due_date, actual_delivery_date.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Their field</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Our source</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Rule</t>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>CANCEL/RETURNS</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>⚠️</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>No cancel or returns API (outbound cancel unsupported on our side anyway).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>profile.first_name / last_name</t>
+          <t>CATALOG</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>shipping_firstname / shipping_lastname</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Empty last name uses first name (required). Shipping has no name field, so profile is the recipient.</t>
+          <t>product_listing (total, no paging) + product_details per product (selector undocumented). No price, brand or stock. sku = {product_id}_{size_id}.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
+          <t>BALANCE</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>➖</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>None. No karma_reports module needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Endpoints</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Operation</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>GET ?method=generate_token&amp;corporate_id={id}</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Headers client-secret, client-id, user-name. TTL not documented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Place order</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>POST ?method=order</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>profile, product, shipping (or location code), billing code. 200 orders_id; 409 {orders:[ids]} keyed on user; 400/401/500.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Track order</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>POST ?method=order_status&amp;orders_id={id}</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>orders_status (same field our polling reads), tracking_number, tracking_url, shipping_company, due and delivery dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>POST ?method=product_listing</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>total + data[product_id, name, status]. No paging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Product details</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>POST ?method=product_details</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Selector not documented (assume &amp;product_id=). Sizes, templates, images, GST, HSN. No price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>POST ?method=category_listing</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Category names for products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Create user</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>POST ?method=create_user&amp;...</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>All data in the URL query. Only needed if orders require an existing user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Order field mapping</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Their field</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Our source</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>profile.first_name / last_name</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>shipping_firstname / shipping_lastname</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Empty last name uses first name (required). Shipping has no name field, so profile is the recipient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
           <t>profile.mobile_number</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>shipping_contact_no or recipientMobileNumber</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>Digits only, last 10 for India (assumption).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>profile.email</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Constant order email (Model A)</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Pending Q3: per-user limits would reject repeat orders.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>profile.company_name / corporate_id</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>Config constants</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>Required.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>profile.reference_number</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>externalOrderId</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Always sent; not echoed or searchable.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>product.product_id / size_id</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>sku "{product_id}_{size_id}"</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Split; omit size_id when absent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>shipping.address_line_1 / 2, city, state, pincode</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>shipping_address_1 / 2, shipping_city, shipping_zone, shipping_postcode</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>State as name; pincode as text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>shipping.country</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>shipping country</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>99 = India; block other countries until confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>corporate_billing_id</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Config constant</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Location code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Status flow</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Their status</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Our status</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>What happens</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>in production (10)</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>CONFIRMED</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Delivery record created; status email.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>dispatched? (not documented)</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>SHIPPED</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>Courier tracking saved; email.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>delivered? (not documented)</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>DELIVERED</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Final; status checks stop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>cancelled / rejected? (not documented)</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>CANCELED</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>Refund queued; status checks stop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>returned? (not documented)</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>RETURNED</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Email only, no refund; status checks continue (not terminal).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>anything else</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>(unmapped)</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>Tracking only; logged as unmapped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Failure modes</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>Failure</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Handling</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Severity</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Timeout or 5xx after Printstop created the order</t>
+          <t>shipping.address_line_1 / 2, city, state, pincode</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>No automatic retry (no lookup by reference); manual reconcile.</t>
+          <t>shipping_address_1 / 2, shipping_city, shipping_zone, shipping_postcode</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>State as name; pincode as text.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>409 duplicate returns another reward's order (same user)</t>
+          <t>shipping.country</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Never link automatically; manual review.</t>
+          <t>shipping country</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>99 = India; block other countries until confirmed.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>One status call fails</t>
+          <t>corporate_billing_id</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Must not stop status checks for all other orders.</t>
+          <t>Config constant</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>Status email re-sent on every check (suspected base bug)</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>Verify before go-live; this vendor relies only on status checks.</t>
-        </is>
-      </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Location code.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue detail call fails mid-sync</t>
-        </is>
-      </c>
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>Throw so the sync never wipes the catalogue with partial data.</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Status flow</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>Token expires or secret rotated</t>
-        </is>
-      </c>
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t>Refresh every 30 min until TTL is known; alert on refresh failure.</t>
-        </is>
-      </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Their status</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Our status</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>What happens</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Unmapped status</t>
+          <t>in production (10)</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Alert; add to status map.</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Delivery record created; status email.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Order stuck or returned, never final</t>
+          <t>dispatched? (not documented)</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Ageing alert past due date + 7 days.</t>
+          <t>SHIPPED</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Courier tracking saved; email.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>Personalised product ordered without template</t>
+          <t>delivered? (not documented)</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Disabled at sync.</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Final; status checks stop.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Price differs from our stored amount</t>
+          <t>cancelled / rejected? (not documented)</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Keep karma amounts in sync; ask for a price field.</t>
+          <t>CANCELED</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Refund queued; status checks stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>returned? (not documented)</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>RETURNED</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Email only, no refund; status checks continue (not terminal).</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Assumptions to verify</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>How to verify</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr"/>
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>anything else</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>(unmapped)</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Tracking only; logged as unmapped.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
-        <is>
-          <t>Token lasts about 1 hour (Firebase default)</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>Ask; decode exp in a sandbox token.</t>
-        </is>
-      </c>
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Failure modes</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n"/>
+      <c r="C53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>product_details takes &amp;product_id=</t>
-        </is>
-      </c>
-      <c r="B54" s="10" t="inlineStr">
-        <is>
-          <t>Sandbox request.</t>
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Failure</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Handling</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Severity</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Status list has dispatched, delivered, cancelled, returned equivalents</t>
+          <t>Timeout or 5xx after Printstop created the order</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>Vendor question 1.</t>
+          <t>No automatic retry (no lookup by reference); manual reconcile.</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Indian mobile numbers accepted as 10 digits</t>
+          <t>409 duplicate returns another reward's order (same user)</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Sandbox orders with different formats.</t>
+          <t>Never link automatically; manual review.</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>Dates are IST; orders_date_finished is the order date</t>
+          <t>One status call fails</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>Ask Printstop.</t>
+          <t>Must not stop status checks for all other orders.</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Sandbox orders are not shipped or billed</t>
+          <t>Status email re-sent on every check (suspected base bug)</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Ask before the first sandbox order.</t>
+          <t>Verify before go-live; this vendor relies only on status checks.</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>Our base code's polling loop stops on a thrown error</t>
+          <t>Catalogue detail call fails mid-sync</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>Read vendorMerchandiseClass on the branch.</t>
+          <t>Throw so the sync never wipes the catalogue with partial data.</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Token expires or secret rotated</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Refresh every 30 min until TTL is known; alert on refresh failure.</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>Config changes</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="n"/>
-      <c r="C61" s="3" t="n"/>
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>Unmapped status</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>Alert; add to status map.</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr"/>
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>Order stuck or returned, never final</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>Ageing alert past due date + 7 days.</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>VI vendorConfigs/Printstop.json</t>
+          <t>Personalised product ordered without template</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>merchandiseVendor true, iswebhookConfiration true, fixedSku + skuTable, token/refetch/listing blocks, credentials under one key "printstop".</t>
+          <t>Disabled at sync.</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
+          <t>Price differs from our stored amount</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Keep karma amounts in sync; ask for a price field.</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Assumptions to verify</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>How to verify</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>Token lasts about 1 hour (Firebase default)</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>Ask; decode exp in a sandbox token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>product_details takes &amp;product_id=</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Sandbox request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>Status list has dispatched, delivered, cancelled, returned equivalents</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>Vendor question 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Indian mobile numbers accepted as 10 digits</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Sandbox orders with different formats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>Dates are IST; orders_date_finished is the order date</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>Ask Printstop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Sandbox orders are not shipped or billed</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Ask before the first sandbox order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>Our base code's polling loop stops on a thrown error</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>Read vendorMerchandiseClass on the branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Config changes</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="n"/>
+      <c r="C76" s="3" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>VI vendorConfigs/Printstop.json</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>merchandiseVendor true, iswebhookConfiration true, fixedSku + skuTable, token/refetch/listing blocks, credentials under one key "printstop".</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
           <t>VI baseConfigs</t>
         </is>
       </c>
-      <c r="B64" s="10" t="inlineStr">
+      <c r="B79" s="10" t="inlineStr">
         <is>
           <t>vendorClassIdMapping, merchandiseOrderTrackingVendorIds, redactHeaders (client-secret, client-id, user-name), allowMerchandiseEmailClientIds if Plum Pro.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="9" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>OPMS</t>
         </is>
       </c>
-      <c r="B65" s="9" t="inlineStr">
+      <c r="B80" s="9" t="inlineStr">
         <is>
           <t>integratedVendors += "&lt;id&gt;" (string).</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="10" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
         <is>
           <t>Schedulers</t>
         </is>
       </c>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="B81" s="10" t="inlineStr">
         <is>
           <t>Token refresh every 30 min, catalogue sync daily, status checks every 30-60 min.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="9" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="9" t="inlineStr">
         <is>
           <t>DB / karma</t>
         </is>
       </c>
-      <c r="B67" s="9" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>Check existing Printstop rows, tables and admin pages first; add only what is missing.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>Build notes</t>
         </is>
       </c>
-      <c r="B69" s="3" t="n"/>
-      <c r="C69" s="3" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="3" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
         <is>
           <t>- Check first: karma already defines PRINTSTPMERCHANDISE_VENDOR_ID, so a connector may exist.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
         <is>
           <t>- Status checks need no override: their field is orders_status, which our polling already reads.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
         <is>
           <t>- No webhooks: nothing to add in plumAuth. No balance API: no karma_reports module.</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="12" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
         <is>
           <t>- Full developer spec: Printstop_TECH_SPEC.md.</t>
         </is>
@@ -4256,11 +4486,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A85:C85"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A88:C88"/>
+    <mergeCell ref="A87:C87"/>
+    <mergeCell ref="A86:C86"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>